<commit_message>
Remove the trunk/proboscis filter
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/animals.xlsx
+++ b/data/animals.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Lists" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Animals'!$A$1:$V$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Animals'!$A$1:$U$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V201"/>
+  <dimension ref="A1:U201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,6 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -678,11 +677,6 @@
           <t>Has snout</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
-        <is>
-          <t>Has trunk</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -760,7 +754,6 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -842,7 +835,6 @@
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -924,7 +916,6 @@
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1006,7 +997,6 @@
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1088,7 +1078,6 @@
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1170,7 +1159,6 @@
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1248,11 +1236,6 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1334,7 +1317,6 @@
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1416,7 +1398,6 @@
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1494,7 +1475,6 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1576,7 +1556,6 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1658,7 +1637,6 @@
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1740,7 +1718,6 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1822,7 +1799,6 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1900,7 +1876,6 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1978,7 +1953,6 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2056,7 +2030,6 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2134,7 +2107,6 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2212,7 +2184,6 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2290,7 +2261,6 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2368,7 +2338,6 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2450,7 +2419,6 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2532,7 +2500,6 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2610,7 +2577,6 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2692,7 +2658,6 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2774,7 +2739,6 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2856,7 +2820,6 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2934,7 +2897,6 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3012,7 +2974,6 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3090,7 +3051,6 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3172,7 +3132,6 @@
       </c>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3258,7 +3217,6 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3340,7 +3298,6 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3418,7 +3375,6 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3496,7 +3452,6 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3574,7 +3529,6 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3652,7 +3606,6 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3726,7 +3679,6 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3804,7 +3756,6 @@
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3878,7 +3829,6 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3952,7 +3902,6 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4038,7 +3987,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4124,7 +4072,6 @@
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
-      <c r="V44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4210,11 +4157,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4300,7 +4242,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4378,7 +4319,6 @@
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4460,7 +4400,6 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4546,7 +4485,6 @@
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4628,7 +4566,6 @@
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4714,7 +4651,6 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4796,7 +4732,6 @@
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4878,7 +4813,6 @@
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
-      <c r="V53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4960,7 +4894,6 @@
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5042,7 +4975,6 @@
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5128,7 +5060,6 @@
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr"/>
-      <c r="V56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5210,7 +5141,6 @@
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr"/>
       <c r="U57" t="inlineStr"/>
-      <c r="V57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5292,7 +5222,6 @@
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr"/>
-      <c r="V58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5374,7 +5303,6 @@
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
-      <c r="V59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5456,7 +5384,6 @@
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
-      <c r="V60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5542,7 +5469,6 @@
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr"/>
-      <c r="V61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5628,7 +5554,6 @@
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
-      <c r="V62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5714,7 +5639,6 @@
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5792,7 +5716,6 @@
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5878,7 +5801,6 @@
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5964,7 +5886,6 @@
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr"/>
       <c r="U66" t="inlineStr"/>
-      <c r="V66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6046,7 +5967,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6128,7 +6048,6 @@
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6210,7 +6129,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6288,7 +6206,6 @@
       <c r="S70" t="inlineStr"/>
       <c r="T70" t="inlineStr"/>
       <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6366,7 +6283,6 @@
       <c r="S71" t="inlineStr"/>
       <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr"/>
-      <c r="V71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6444,7 +6360,6 @@
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr"/>
-      <c r="V72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6522,7 +6437,6 @@
       <c r="S73" t="inlineStr"/>
       <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6608,7 +6522,6 @@
         </is>
       </c>
       <c r="U74" t="inlineStr"/>
-      <c r="V74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6686,7 +6599,6 @@
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr"/>
-      <c r="V75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6768,7 +6680,6 @@
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr"/>
-      <c r="V76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6850,7 +6761,6 @@
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr"/>
-      <c r="V77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6928,7 +6838,6 @@
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr"/>
-      <c r="V78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7002,7 +6911,6 @@
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr"/>
       <c r="U79" t="inlineStr"/>
-      <c r="V79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7080,7 +6988,6 @@
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr"/>
       <c r="U80" t="inlineStr"/>
-      <c r="V80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7166,7 +7073,6 @@
         </is>
       </c>
       <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7244,7 +7150,6 @@
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr"/>
-      <c r="V82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7326,7 +7231,6 @@
         </is>
       </c>
       <c r="U83" t="inlineStr"/>
-      <c r="V83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7404,7 +7308,6 @@
       <c r="S84" t="inlineStr"/>
       <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr"/>
-      <c r="V84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7478,7 +7381,6 @@
       <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7560,7 +7462,6 @@
       <c r="S86" t="inlineStr"/>
       <c r="T86" t="inlineStr"/>
       <c r="U86" t="inlineStr"/>
-      <c r="V86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7642,7 +7543,6 @@
         </is>
       </c>
       <c r="U87" t="inlineStr"/>
-      <c r="V87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7720,7 +7620,6 @@
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr"/>
-      <c r="V88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7806,7 +7705,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7888,7 +7786,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7966,7 +7863,6 @@
       <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr"/>
       <c r="U91" t="inlineStr"/>
-      <c r="V91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8048,7 +7944,6 @@
       </c>
       <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr"/>
-      <c r="V92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8126,7 +8021,6 @@
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
-      <c r="V93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8208,7 +8102,6 @@
       <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr"/>
-      <c r="V94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8290,7 +8183,6 @@
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="inlineStr"/>
       <c r="U95" t="inlineStr"/>
-      <c r="V95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8372,7 +8264,6 @@
       <c r="S96" t="inlineStr"/>
       <c r="T96" t="inlineStr"/>
       <c r="U96" t="inlineStr"/>
-      <c r="V96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8454,7 +8345,6 @@
       </c>
       <c r="T97" t="inlineStr"/>
       <c r="U97" t="inlineStr"/>
-      <c r="V97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8540,7 +8430,6 @@
         </is>
       </c>
       <c r="U98" t="inlineStr"/>
-      <c r="V98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8618,7 +8507,6 @@
       <c r="S99" t="inlineStr"/>
       <c r="T99" t="inlineStr"/>
       <c r="U99" t="inlineStr"/>
-      <c r="V99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8692,7 +8580,6 @@
       <c r="S100" t="inlineStr"/>
       <c r="T100" t="inlineStr"/>
       <c r="U100" t="inlineStr"/>
-      <c r="V100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8774,7 +8661,6 @@
       <c r="S101" t="inlineStr"/>
       <c r="T101" t="inlineStr"/>
       <c r="U101" t="inlineStr"/>
-      <c r="V101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8852,11 +8738,6 @@
       <c r="S102" t="inlineStr"/>
       <c r="T102" t="inlineStr"/>
       <c r="U102" t="inlineStr"/>
-      <c r="V102" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8930,7 +8811,6 @@
       <c r="S103" t="inlineStr"/>
       <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr"/>
-      <c r="V103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9008,7 +8888,6 @@
       <c r="S104" t="inlineStr"/>
       <c r="T104" t="inlineStr"/>
       <c r="U104" t="inlineStr"/>
-      <c r="V104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9090,7 +8969,6 @@
       <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr"/>
-      <c r="V105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -9172,7 +9050,6 @@
       <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr"/>
       <c r="U106" t="inlineStr"/>
-      <c r="V106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -9246,7 +9123,6 @@
       <c r="S107" t="inlineStr"/>
       <c r="T107" t="inlineStr"/>
       <c r="U107" t="inlineStr"/>
-      <c r="V107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9324,7 +9200,6 @@
       <c r="S108" t="inlineStr"/>
       <c r="T108" t="inlineStr"/>
       <c r="U108" t="inlineStr"/>
-      <c r="V108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9398,7 +9273,6 @@
       <c r="S109" t="inlineStr"/>
       <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr"/>
-      <c r="V109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9472,7 +9346,6 @@
       <c r="S110" t="inlineStr"/>
       <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr"/>
-      <c r="V110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9546,7 +9419,6 @@
       <c r="S111" t="inlineStr"/>
       <c r="T111" t="inlineStr"/>
       <c r="U111" t="inlineStr"/>
-      <c r="V111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9620,7 +9492,6 @@
       <c r="S112" t="inlineStr"/>
       <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr"/>
-      <c r="V112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9698,11 +9569,6 @@
       <c r="S113" t="inlineStr"/>
       <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
-      <c r="V113" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9780,7 +9646,6 @@
       <c r="S114" t="inlineStr"/>
       <c r="T114" t="inlineStr"/>
       <c r="U114" t="inlineStr"/>
-      <c r="V114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9858,7 +9723,6 @@
       <c r="S115" t="inlineStr"/>
       <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr"/>
-      <c r="V115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9940,7 +9804,6 @@
         </is>
       </c>
       <c r="U116" t="inlineStr"/>
-      <c r="V116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -10018,7 +9881,6 @@
       <c r="S117" t="inlineStr"/>
       <c r="T117" t="inlineStr"/>
       <c r="U117" t="inlineStr"/>
-      <c r="V117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -10096,7 +9958,6 @@
       <c r="S118" t="inlineStr"/>
       <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr"/>
-      <c r="V118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -10174,7 +10035,6 @@
       <c r="S119" t="inlineStr"/>
       <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr"/>
-      <c r="V119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -10256,7 +10116,6 @@
         </is>
       </c>
       <c r="U120" t="inlineStr"/>
-      <c r="V120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -10338,7 +10197,6 @@
       <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
-      <c r="V121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -10420,7 +10278,6 @@
       <c r="S122" t="inlineStr"/>
       <c r="T122" t="inlineStr"/>
       <c r="U122" t="inlineStr"/>
-      <c r="V122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -10502,7 +10359,6 @@
       <c r="S123" t="inlineStr"/>
       <c r="T123" t="inlineStr"/>
       <c r="U123" t="inlineStr"/>
-      <c r="V123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -10584,7 +10440,6 @@
       </c>
       <c r="T124" t="inlineStr"/>
       <c r="U124" t="inlineStr"/>
-      <c r="V124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -10662,7 +10517,6 @@
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr"/>
       <c r="U125" t="inlineStr"/>
-      <c r="V125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -10740,7 +10594,6 @@
       <c r="S126" t="inlineStr"/>
       <c r="T126" t="inlineStr"/>
       <c r="U126" t="inlineStr"/>
-      <c r="V126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -10826,7 +10679,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -10908,7 +10760,6 @@
       <c r="S128" t="inlineStr"/>
       <c r="T128" t="inlineStr"/>
       <c r="U128" t="inlineStr"/>
-      <c r="V128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10986,7 +10837,6 @@
       <c r="S129" t="inlineStr"/>
       <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr"/>
-      <c r="V129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -11068,7 +10918,6 @@
       <c r="S130" t="inlineStr"/>
       <c r="T130" t="inlineStr"/>
       <c r="U130" t="inlineStr"/>
-      <c r="V130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -11146,7 +10995,6 @@
       <c r="S131" t="inlineStr"/>
       <c r="T131" t="inlineStr"/>
       <c r="U131" t="inlineStr"/>
-      <c r="V131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -11228,7 +11076,6 @@
       <c r="S132" t="inlineStr"/>
       <c r="T132" t="inlineStr"/>
       <c r="U132" t="inlineStr"/>
-      <c r="V132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -11306,7 +11153,6 @@
       <c r="S133" t="inlineStr"/>
       <c r="T133" t="inlineStr"/>
       <c r="U133" t="inlineStr"/>
-      <c r="V133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -11388,7 +11234,6 @@
       <c r="S134" t="inlineStr"/>
       <c r="T134" t="inlineStr"/>
       <c r="U134" t="inlineStr"/>
-      <c r="V134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -11470,7 +11315,6 @@
       <c r="S135" t="inlineStr"/>
       <c r="T135" t="inlineStr"/>
       <c r="U135" t="inlineStr"/>
-      <c r="V135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -11552,7 +11396,6 @@
       <c r="S136" t="inlineStr"/>
       <c r="T136" t="inlineStr"/>
       <c r="U136" t="inlineStr"/>
-      <c r="V136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -11634,7 +11477,6 @@
       <c r="S137" t="inlineStr"/>
       <c r="T137" t="inlineStr"/>
       <c r="U137" t="inlineStr"/>
-      <c r="V137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -11712,7 +11554,6 @@
       <c r="S138" t="inlineStr"/>
       <c r="T138" t="inlineStr"/>
       <c r="U138" t="inlineStr"/>
-      <c r="V138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -11794,7 +11635,6 @@
       <c r="S139" t="inlineStr"/>
       <c r="T139" t="inlineStr"/>
       <c r="U139" t="inlineStr"/>
-      <c r="V139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -11872,7 +11712,6 @@
       <c r="S140" t="inlineStr"/>
       <c r="T140" t="inlineStr"/>
       <c r="U140" t="inlineStr"/>
-      <c r="V140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -11950,7 +11789,6 @@
       <c r="S141" t="inlineStr"/>
       <c r="T141" t="inlineStr"/>
       <c r="U141" t="inlineStr"/>
-      <c r="V141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -12028,7 +11866,6 @@
       <c r="S142" t="inlineStr"/>
       <c r="T142" t="inlineStr"/>
       <c r="U142" t="inlineStr"/>
-      <c r="V142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -12110,7 +11947,6 @@
       </c>
       <c r="T143" t="inlineStr"/>
       <c r="U143" t="inlineStr"/>
-      <c r="V143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -12188,7 +12024,6 @@
       <c r="S144" t="inlineStr"/>
       <c r="T144" t="inlineStr"/>
       <c r="U144" t="inlineStr"/>
-      <c r="V144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -12262,7 +12097,6 @@
       <c r="S145" t="inlineStr"/>
       <c r="T145" t="inlineStr"/>
       <c r="U145" t="inlineStr"/>
-      <c r="V145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -12344,7 +12178,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -12422,7 +12255,6 @@
       <c r="S147" t="inlineStr"/>
       <c r="T147" t="inlineStr"/>
       <c r="U147" t="inlineStr"/>
-      <c r="V147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -12504,7 +12336,6 @@
       <c r="S148" t="inlineStr"/>
       <c r="T148" t="inlineStr"/>
       <c r="U148" t="inlineStr"/>
-      <c r="V148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -12586,7 +12417,6 @@
       <c r="S149" t="inlineStr"/>
       <c r="T149" t="inlineStr"/>
       <c r="U149" t="inlineStr"/>
-      <c r="V149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -12668,7 +12498,6 @@
       <c r="S150" t="inlineStr"/>
       <c r="T150" t="inlineStr"/>
       <c r="U150" t="inlineStr"/>
-      <c r="V150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -12750,7 +12579,6 @@
       <c r="S151" t="inlineStr"/>
       <c r="T151" t="inlineStr"/>
       <c r="U151" t="inlineStr"/>
-      <c r="V151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -12832,7 +12660,6 @@
       <c r="S152" t="inlineStr"/>
       <c r="T152" t="inlineStr"/>
       <c r="U152" t="inlineStr"/>
-      <c r="V152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -12914,7 +12741,6 @@
       <c r="S153" t="inlineStr"/>
       <c r="T153" t="inlineStr"/>
       <c r="U153" t="inlineStr"/>
-      <c r="V153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -12996,7 +12822,6 @@
       <c r="S154" t="inlineStr"/>
       <c r="T154" t="inlineStr"/>
       <c r="U154" t="inlineStr"/>
-      <c r="V154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -13078,7 +12903,6 @@
       <c r="S155" t="inlineStr"/>
       <c r="T155" t="inlineStr"/>
       <c r="U155" t="inlineStr"/>
-      <c r="V155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -13164,7 +12988,6 @@
       <c r="S156" t="inlineStr"/>
       <c r="T156" t="inlineStr"/>
       <c r="U156" t="inlineStr"/>
-      <c r="V156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -13250,7 +13073,6 @@
       <c r="S157" t="inlineStr"/>
       <c r="T157" t="inlineStr"/>
       <c r="U157" t="inlineStr"/>
-      <c r="V157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -13332,7 +13154,6 @@
       <c r="S158" t="inlineStr"/>
       <c r="T158" t="inlineStr"/>
       <c r="U158" t="inlineStr"/>
-      <c r="V158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -13418,7 +13239,6 @@
       <c r="S159" t="inlineStr"/>
       <c r="T159" t="inlineStr"/>
       <c r="U159" t="inlineStr"/>
-      <c r="V159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -13504,7 +13324,6 @@
       <c r="S160" t="inlineStr"/>
       <c r="T160" t="inlineStr"/>
       <c r="U160" t="inlineStr"/>
-      <c r="V160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -13582,7 +13401,6 @@
       <c r="S161" t="inlineStr"/>
       <c r="T161" t="inlineStr"/>
       <c r="U161" t="inlineStr"/>
-      <c r="V161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -13656,7 +13474,6 @@
       <c r="S162" t="inlineStr"/>
       <c r="T162" t="inlineStr"/>
       <c r="U162" t="inlineStr"/>
-      <c r="V162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -13738,7 +13555,6 @@
       <c r="S163" t="inlineStr"/>
       <c r="T163" t="inlineStr"/>
       <c r="U163" t="inlineStr"/>
-      <c r="V163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -13824,7 +13640,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -13906,7 +13721,6 @@
         </is>
       </c>
       <c r="U165" t="inlineStr"/>
-      <c r="V165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -13984,7 +13798,6 @@
       <c r="S166" t="inlineStr"/>
       <c r="T166" t="inlineStr"/>
       <c r="U166" t="inlineStr"/>
-      <c r="V166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -14062,7 +13875,6 @@
       <c r="S167" t="inlineStr"/>
       <c r="T167" t="inlineStr"/>
       <c r="U167" t="inlineStr"/>
-      <c r="V167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -14148,7 +13960,6 @@
         </is>
       </c>
       <c r="U168" t="inlineStr"/>
-      <c r="V168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -14230,7 +14041,6 @@
         </is>
       </c>
       <c r="U169" t="inlineStr"/>
-      <c r="V169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -14312,7 +14122,6 @@
       <c r="S170" t="inlineStr"/>
       <c r="T170" t="inlineStr"/>
       <c r="U170" t="inlineStr"/>
-      <c r="V170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -14394,7 +14203,6 @@
       </c>
       <c r="T171" t="inlineStr"/>
       <c r="U171" t="inlineStr"/>
-      <c r="V171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -14472,7 +14280,6 @@
       <c r="S172" t="inlineStr"/>
       <c r="T172" t="inlineStr"/>
       <c r="U172" t="inlineStr"/>
-      <c r="V172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -14550,7 +14357,6 @@
       <c r="S173" t="inlineStr"/>
       <c r="T173" t="inlineStr"/>
       <c r="U173" t="inlineStr"/>
-      <c r="V173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -14632,7 +14438,6 @@
         </is>
       </c>
       <c r="U174" t="inlineStr"/>
-      <c r="V174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -14710,7 +14515,6 @@
       <c r="S175" t="inlineStr"/>
       <c r="T175" t="inlineStr"/>
       <c r="U175" t="inlineStr"/>
-      <c r="V175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -14784,7 +14588,6 @@
       <c r="S176" t="inlineStr"/>
       <c r="T176" t="inlineStr"/>
       <c r="U176" t="inlineStr"/>
-      <c r="V176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -14862,7 +14665,6 @@
       <c r="S177" t="inlineStr"/>
       <c r="T177" t="inlineStr"/>
       <c r="U177" t="inlineStr"/>
-      <c r="V177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -14944,7 +14746,6 @@
       <c r="S178" t="inlineStr"/>
       <c r="T178" t="inlineStr"/>
       <c r="U178" t="inlineStr"/>
-      <c r="V178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -15026,7 +14827,6 @@
       <c r="S179" t="inlineStr"/>
       <c r="T179" t="inlineStr"/>
       <c r="U179" t="inlineStr"/>
-      <c r="V179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -15108,7 +14908,6 @@
       <c r="S180" t="inlineStr"/>
       <c r="T180" t="inlineStr"/>
       <c r="U180" t="inlineStr"/>
-      <c r="V180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -15182,7 +14981,6 @@
       <c r="S181" t="inlineStr"/>
       <c r="T181" t="inlineStr"/>
       <c r="U181" t="inlineStr"/>
-      <c r="V181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -15264,7 +15062,6 @@
       <c r="S182" t="inlineStr"/>
       <c r="T182" t="inlineStr"/>
       <c r="U182" t="inlineStr"/>
-      <c r="V182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -15342,7 +15139,6 @@
       <c r="S183" t="inlineStr"/>
       <c r="T183" t="inlineStr"/>
       <c r="U183" t="inlineStr"/>
-      <c r="V183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -15420,7 +15216,6 @@
       <c r="S184" t="inlineStr"/>
       <c r="T184" t="inlineStr"/>
       <c r="U184" t="inlineStr"/>
-      <c r="V184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -15506,7 +15301,6 @@
       </c>
       <c r="T185" t="inlineStr"/>
       <c r="U185" t="inlineStr"/>
-      <c r="V185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -15588,7 +15382,6 @@
         </is>
       </c>
       <c r="U186" t="inlineStr"/>
-      <c r="V186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -15666,7 +15459,6 @@
       <c r="S187" t="inlineStr"/>
       <c r="T187" t="inlineStr"/>
       <c r="U187" t="inlineStr"/>
-      <c r="V187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -15752,7 +15544,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="V188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -15834,7 +15625,6 @@
       <c r="S189" t="inlineStr"/>
       <c r="T189" t="inlineStr"/>
       <c r="U189" t="inlineStr"/>
-      <c r="V189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -15912,7 +15702,6 @@
       <c r="S190" t="inlineStr"/>
       <c r="T190" t="inlineStr"/>
       <c r="U190" t="inlineStr"/>
-      <c r="V190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -15986,7 +15775,6 @@
       <c r="S191" t="inlineStr"/>
       <c r="T191" t="inlineStr"/>
       <c r="U191" t="inlineStr"/>
-      <c r="V191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -16064,7 +15852,6 @@
       <c r="S192" t="inlineStr"/>
       <c r="T192" t="inlineStr"/>
       <c r="U192" t="inlineStr"/>
-      <c r="V192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -16142,7 +15929,6 @@
       <c r="S193" t="inlineStr"/>
       <c r="T193" t="inlineStr"/>
       <c r="U193" t="inlineStr"/>
-      <c r="V193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -16220,7 +16006,6 @@
       <c r="S194" t="inlineStr"/>
       <c r="T194" t="inlineStr"/>
       <c r="U194" t="inlineStr"/>
-      <c r="V194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -16294,7 +16079,6 @@
       <c r="S195" t="inlineStr"/>
       <c r="T195" t="inlineStr"/>
       <c r="U195" t="inlineStr"/>
-      <c r="V195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -16372,7 +16156,6 @@
       <c r="S196" t="inlineStr"/>
       <c r="T196" t="inlineStr"/>
       <c r="U196" t="inlineStr"/>
-      <c r="V196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -16450,7 +16233,6 @@
       <c r="S197" t="inlineStr"/>
       <c r="T197" t="inlineStr"/>
       <c r="U197" t="inlineStr"/>
-      <c r="V197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -16528,11 +16310,6 @@
       <c r="S198" t="inlineStr"/>
       <c r="T198" t="inlineStr"/>
       <c r="U198" t="inlineStr"/>
-      <c r="V198" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -16606,7 +16383,6 @@
       <c r="S199" t="inlineStr"/>
       <c r="T199" t="inlineStr"/>
       <c r="U199" t="inlineStr"/>
-      <c r="V199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -16684,7 +16460,6 @@
       <c r="S200" t="inlineStr"/>
       <c r="T200" t="inlineStr"/>
       <c r="U200" t="inlineStr"/>
-      <c r="V200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -16762,11 +16537,10 @@
       <c r="S201" t="inlineStr"/>
       <c r="T201" t="inlineStr"/>
       <c r="U201" t="inlineStr"/>
-      <c r="V201" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V201"/>
-  <dataValidations count="19">
+  <autoFilter ref="A1:U201"/>
+  <dataValidations count="18">
     <dataValidation sqref="C2:C700" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Lists!$A$2:$A$7</formula1>
     </dataValidation>
@@ -16822,9 +16596,6 @@
     <dataValidation sqref="U2:U700" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Yes"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V700" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Yes"</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>